<commit_message>
Add 1/2in ball valve flow comparison to The Squeezer description
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kx49kLBqd9ASW1mJT4wUBP
</commit_message>
<xml_diff>
--- a/washdown/Washdown_Long_Descriptions_Review.xlsx
+++ b/washdown/Washdown_Long_Descriptions_Review.xlsx
@@ -409,10 +409,10 @@
     <t xml:space="preserve">Self-closing valve for liquids and foam. Takes hoses, lances and nozzles.</t>
   </si>
   <si>
-    <t xml:space="preserve">The Squeezer is a self-closing valve: squeeze to open, and the flow stops as soon as you let go. It works with water, other liquids and foam, and takes hoses, lances and nozzles, so it can be the base of many different cleaning and dosing setups. It's made from AISI 304 stainless and rated to 40 bar and 95°C, with around 57 l/min of flow. Fit the Squeezer Shower Head to turn it into a soft-wash tool for delicate produce.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Dosing setups" is suggested from "liquids and foam".</t>
+    <t xml:space="preserve">The Squeezer is a self-closing valve: squeeze to open, and the flow stops as soon as you let go. It works with water, other liquids and foam, and takes hoses, lances and nozzles, so it can be the base of many different cleaning and dosing setups. It's made from AISI 304 stainless and rated to 40 bar and 95°C, with around 57 l/min of flow. That's flow capacity comparable to a 1/2" ball valve, so it can take the place of one without reducing supply. Fit the Squeezer Shower Head to turn it into a soft-wash tool for delicate produce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Dosing setups" is suggested from "liquids and foam". The 1/2\" ball valve comparison was added at your request; "without reducing supply" is my wording.</t>
   </si>
   <si>
     <t xml:space="preserve">the-squeezer</t>
@@ -1655,7 +1655,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="F27" s="4" t="n">
         <f aca="false">IF(LEN(TRIM(E27))=0,0,LEN(TRIM(E27))-LEN(SUBSTITUTE(TRIM(E27)," ",""))+1)</f>
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G27" s="4" t="s">
         <v>129</v>

</xml_diff>